<commit_message>
修正def addDataframe_index(df1, df2):     index = df2.index     if index[0]:         for i in index:             df1.loc['第8天', :][i] = df1.loc['第8天', :][i] + s[i]     else:         print("今日pca没有新单")
</commit_message>
<xml_diff>
--- a/新开户均/新开部门行业户均监控表.xlsx
+++ b/新开户均/新开部门行业户均监控表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="8010" activeTab="1"/>
+    <workbookView windowWidth="20490" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="明细" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="80">
   <si>
     <t>大区</t>
   </si>
@@ -56,97 +56,94 @@
     <t>户均完成率</t>
   </si>
   <si>
-    <t>搜索点击消费20230801</t>
+    <t>搜索点击消费20230901</t>
   </si>
   <si>
-    <t>搜索点击消费20230802</t>
+    <t>搜索点击消费20230902</t>
   </si>
   <si>
-    <t>搜索点击消费20230803</t>
+    <t>搜索点击消费20230903</t>
   </si>
   <si>
-    <t>搜索点击消费20230804</t>
+    <t>搜索点击消费20230904</t>
   </si>
   <si>
-    <t>搜索点击消费20230805</t>
+    <t>搜索点击消费20230905</t>
   </si>
   <si>
-    <t>搜索点击消费20230806</t>
+    <t>搜索点击消费20230906</t>
   </si>
   <si>
-    <t>搜索点击消费20230807</t>
+    <t>搜索点击消费20230907</t>
   </si>
   <si>
-    <t>搜索点击消费20230808</t>
+    <t>搜索点击消费20230908</t>
   </si>
   <si>
-    <t>搜索点击消费20230809</t>
+    <t>搜索点击消费20230909</t>
   </si>
   <si>
-    <t>搜索点击消费20230810</t>
+    <t>搜索点击消费20230910</t>
   </si>
   <si>
-    <t>搜索点击消费20230811</t>
+    <t>搜索点击消费20230911</t>
   </si>
   <si>
-    <t>搜索点击消费20230812</t>
+    <t>搜索点击消费20230912</t>
   </si>
   <si>
-    <t>搜索点击消费20230813</t>
+    <t>搜索点击消费20230913</t>
   </si>
   <si>
-    <t>搜索点击消费20230814</t>
+    <t>搜索点击消费20230914</t>
   </si>
   <si>
-    <t>搜索点击消费20230815</t>
+    <t>搜索点击消费20230915</t>
   </si>
   <si>
-    <t>搜索点击消费20230816</t>
+    <t>搜索点击消费20230916</t>
   </si>
   <si>
-    <t>搜索点击消费20230817</t>
+    <t>搜索点击消费20230917</t>
   </si>
   <si>
-    <t>搜索点击消费20230818</t>
+    <t>搜索点击消费20230918</t>
   </si>
   <si>
-    <t>搜索点击消费20230819</t>
+    <t>搜索点击消费20230919</t>
   </si>
   <si>
-    <t>搜索点击消费20230820</t>
+    <t>搜索点击消费20230920</t>
   </si>
   <si>
-    <t>搜索点击消费20230821</t>
+    <t>搜索点击消费20230921</t>
   </si>
   <si>
-    <t>搜索点击消费20230822</t>
+    <t>搜索点击消费20230922</t>
   </si>
   <si>
-    <t>搜索点击消费20230823</t>
+    <t>搜索点击消费20230923</t>
   </si>
   <si>
-    <t>搜索点击消费20230824</t>
+    <t>搜索点击消费20230924</t>
   </si>
   <si>
-    <t>搜索点击消费20230825</t>
+    <t>搜索点击消费20230925</t>
   </si>
   <si>
-    <t>搜索点击消费20230826</t>
+    <t>搜索点击消费20230926</t>
   </si>
   <si>
-    <t>搜索点击消费20230827</t>
+    <t>搜索点击消费20230927</t>
   </si>
   <si>
-    <t>搜索点击消费20230828</t>
+    <t>搜索点击消费20230928</t>
   </si>
   <si>
-    <t>搜索点击消费20230829</t>
+    <t>搜索点击消费20230929</t>
   </si>
   <si>
-    <t>搜索点击消费20230830</t>
-  </si>
-  <si>
-    <t>搜索点击消费20230831</t>
+    <t>搜索点击消费20230930</t>
   </si>
   <si>
     <t>部门</t>
@@ -271,12 +268,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="6">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="#,##0_);[Red]\(#,##0\)"/>
-    <numFmt numFmtId="177" formatCode="#,##0_ "/>
+    <numFmt numFmtId="176" formatCode="#,##0_ "/>
+    <numFmt numFmtId="177" formatCode="#,##0_);[Red]\(#,##0\)"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -305,24 +302,39 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color theme="0"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -337,43 +349,12 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="宋体"/>
@@ -389,8 +370,39 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -411,31 +423,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="major"/>
-    </font>
-    <font>
       <b/>
-      <sz val="15"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -450,7 +447,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -462,67 +477,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -540,7 +513,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -552,25 +543,55 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor rgb="FFFFCC99"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -582,43 +603,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -630,7 +627,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -685,32 +682,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
+      <left/>
+      <right/>
       <top style="thin">
-        <color rgb="FFB2B2B2"/>
+        <color theme="4"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -726,11 +704,24 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FFB2B2B2"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -753,8 +744,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.399975585192419"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -762,17 +753,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4" tint="0.399975585192419"/>
       </bottom>
       <diagonal/>
     </border>
@@ -791,6 +773,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -799,10 +796,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -811,136 +808,136 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -993,7 +990,7 @@
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1002,10 +999,10 @@
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="11" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" xfId="8" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1370,7 +1367,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AQ1143"/>
+  <dimension ref="A1:AP1143"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="16" style="2" customWidth="1"/>
@@ -1395,7 +1392,7 @@
     <col min="41" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:43">
+    <row r="1" s="1" customFormat="1" spans="1:42">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1522,9 +1519,6 @@
       <c r="AP1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="1" t="s">
-        <v>42</v>
-      </c>
     </row>
     <row r="2" spans="9:40">
       <c r="I2" s="18"/>
@@ -17026,48 +17020,48 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:13">
       <c r="A1" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>47</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="M1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="L1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="M1" s="3" t="s">
+    </row>
+    <row r="2" customHeight="1" spans="1:13">
+      <c r="A2" s="4" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="2" customHeight="1" spans="1:13">
-      <c r="A2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>52</v>
       </c>
       <c r="D2" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C2,明细!$I:$I,"&gt;0")</f>
@@ -17082,10 +17076,10 @@
         <v>0.00%</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K2" s="5">
         <f>COUNTIFS(明细!$B:$B,各部门完成情况!J2,明细!$J:$J,"&gt;0")</f>
@@ -17103,10 +17097,10 @@
     <row r="3" spans="1:13">
       <c r="A3" s="4"/>
       <c r="B3" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D3" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C3,明细!$I:$I,"&gt;0")</f>
@@ -17121,10 +17115,10 @@
         <v>0.00%</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K3" s="5">
         <f>COUNTIFS(明细!$B:$B,各部门完成情况!J3,明细!$J:$J,"&gt;0")</f>
@@ -17142,10 +17136,10 @@
     <row r="4" spans="1:13">
       <c r="A4" s="4"/>
       <c r="B4" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D4" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C4,明细!$I:$I,"&gt;0")</f>
@@ -17160,10 +17154,10 @@
         <v>0.00%</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K4" s="5">
         <f>COUNTIFS(明细!$B:$B,各部门完成情况!J4,明细!$J:$J,"&gt;0")</f>
@@ -17181,10 +17175,10 @@
     <row r="5" spans="1:13">
       <c r="A5" s="4"/>
       <c r="B5" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C5,明细!$I:$I,"&gt;0")</f>
@@ -17199,10 +17193,10 @@
         <v>0.00%</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K5" s="5">
         <f>COUNTIFS(明细!$B:$B,各部门完成情况!J5,明细!$J:$J,"&gt;0")</f>
@@ -17220,10 +17214,10 @@
     <row r="6" spans="1:13">
       <c r="A6" s="4"/>
       <c r="B6" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D6" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C6,明细!$I:$I,"&gt;0")</f>
@@ -17246,10 +17240,10 @@
     <row r="7" spans="1:6">
       <c r="A7" s="4"/>
       <c r="B7" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D7" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C7,明细!$I:$I,"&gt;0")</f>
@@ -17267,10 +17261,10 @@
     <row r="8" spans="1:6">
       <c r="A8" s="4"/>
       <c r="B8" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D8" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C8,明细!$I:$I,"&gt;0")</f>
@@ -17288,10 +17282,10 @@
     <row r="9" spans="1:6">
       <c r="A9" s="4"/>
       <c r="B9" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D9" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C9,明细!$I:$I,"&gt;0")</f>
@@ -17309,10 +17303,10 @@
     <row r="10" spans="1:6">
       <c r="A10" s="4"/>
       <c r="B10" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D10" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C10,明细!$I:$I,"&gt;0")</f>
@@ -17330,10 +17324,10 @@
     <row r="11" spans="1:6">
       <c r="A11" s="4"/>
       <c r="B11" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D11" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C11,明细!$I:$I,"&gt;0")</f>
@@ -17351,10 +17345,10 @@
     <row r="12" spans="1:6">
       <c r="A12" s="4"/>
       <c r="B12" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D12" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C12,明细!$I:$I,"&gt;0")</f>
@@ -17372,10 +17366,10 @@
     <row r="13" spans="1:6">
       <c r="A13" s="4"/>
       <c r="B13" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D13" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C13,明细!$I:$I,"&gt;0")</f>
@@ -17393,10 +17387,10 @@
     <row r="14" spans="1:6">
       <c r="A14" s="4"/>
       <c r="B14" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D14" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C14,明细!$I:$I,"&gt;0")</f>
@@ -17413,20 +17407,20 @@
     </row>
     <row r="15" customHeight="1" spans="1:6">
       <c r="A15" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D15" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C15,明细!$I:$I,"&gt;0")</f>
         <v>0</v>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C15,明细!$K:$K,"&gt;=70")</f>
+        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C15,明细!$K:$K,"&gt;=50")</f>
         <v>0</v>
       </c>
       <c r="F15" s="6" t="str">
@@ -17437,17 +17431,17 @@
     <row r="16" customHeight="1" spans="1:6">
       <c r="A16" s="4"/>
       <c r="B16" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D16" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C16,明细!$I:$I,"&gt;0")</f>
         <v>0</v>
       </c>
       <c r="E16" s="5">
-        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C16,明细!$K:$K,"&gt;=70")</f>
+        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C16,明细!$K:$K,"&gt;=50")</f>
         <v>0</v>
       </c>
       <c r="F16" s="6" t="str">
@@ -17458,17 +17452,17 @@
     <row r="17" customHeight="1" spans="1:6">
       <c r="A17" s="4"/>
       <c r="B17" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D17" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C17,明细!$I:$I,"&gt;0")</f>
         <v>0</v>
       </c>
       <c r="E17" s="5">
-        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C17,明细!$K:$K,"&gt;=70")</f>
+        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C17,明细!$K:$K,"&gt;=50")</f>
         <v>0</v>
       </c>
       <c r="F17" s="6" t="str">
@@ -17479,17 +17473,17 @@
     <row r="18" spans="1:6">
       <c r="A18" s="4"/>
       <c r="B18" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D18" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C18,明细!$I:$I,"&gt;0")</f>
         <v>0</v>
       </c>
       <c r="E18" s="5">
-        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C18,明细!$K:$K,"&gt;=70")</f>
+        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C18,明细!$K:$K,"&gt;=50")</f>
         <v>0</v>
       </c>
       <c r="F18" s="6" t="str">
@@ -17500,17 +17494,17 @@
     <row r="19" spans="1:6">
       <c r="A19" s="4"/>
       <c r="B19" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D19" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C19,明细!$I:$I,"&gt;0")</f>
         <v>0</v>
       </c>
       <c r="E19" s="5">
-        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C19,明细!$K:$K,"&gt;=70")</f>
+        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C19,明细!$K:$K,"&gt;=50")</f>
         <v>0</v>
       </c>
       <c r="F19" s="6" t="str">
@@ -17520,20 +17514,20 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D20" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C20,明细!$I:$I,"&gt;0")</f>
         <v>0</v>
       </c>
       <c r="E20" s="5">
-        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C20,明细!$K:$K,"&gt;=70")</f>
+        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C20,明细!$K:$K,"&gt;=50")</f>
         <v>0</v>
       </c>
       <c r="F20" s="6" t="str">
@@ -17544,17 +17538,17 @@
     <row r="21" customHeight="1" spans="1:6">
       <c r="A21" s="10"/>
       <c r="B21" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D21" s="5">
         <f>COUNTIFS(明细!$C:$C,各部门完成情况!C21,明细!$I:$I,"&gt;0")</f>
         <v>0</v>
       </c>
       <c r="E21" s="5">
-        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C21,明细!$K:$K,"&gt;=70")</f>
+        <f>COUNTIFS(明细!$C:$C,各部门完成情况!C21,明细!$K:$K,"&gt;=50")</f>
         <v>0</v>
       </c>
       <c r="F21" s="6" t="str">

</xml_diff>